<commit_message>
Update branding to Tecnoprism M&S, add Sales Team nav, Time & Traceability widget, live Google Sheet sync, and updated master datasets
</commit_message>
<xml_diff>
--- a/public/master/KPI _ Automation COE (2).xlsx
+++ b/public/master/KPI _ Automation COE (2).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="53">
   <si>
     <t>Category</t>
   </si>
@@ -110,6 +110,9 @@
   </si>
   <si>
     <t>478 (268, 210)</t>
+  </si>
+  <si>
+    <t>492 (279, 213)</t>
   </si>
   <si>
     <t>AI Search</t>
@@ -682,7 +685,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="13.75"/>
+    <col customWidth="1" min="1" max="1" width="17.25"/>
     <col customWidth="1" min="2" max="2" width="27.25"/>
     <col customWidth="1" min="3" max="3" width="12.25"/>
     <col customWidth="1" min="10" max="11" width="11.88"/>
@@ -734,7 +737,9 @@
       <c r="O1" s="3">
         <v>46290.0</v>
       </c>
-      <c r="P1" s="5"/>
+      <c r="P1" s="3">
+        <v>46297.0</v>
+      </c>
       <c r="Q1" s="5"/>
       <c r="R1" s="5"/>
       <c r="S1" s="5"/>
@@ -809,7 +814,9 @@
       <c r="O2" s="13">
         <v>399.0</v>
       </c>
-      <c r="P2" s="13"/>
+      <c r="P2" s="13">
+        <v>292.0</v>
+      </c>
       <c r="Q2" s="13"/>
       <c r="R2" s="13"/>
       <c r="S2" s="13"/>
@@ -882,7 +889,9 @@
       <c r="O3" s="13">
         <v>40.0</v>
       </c>
-      <c r="P3" s="13"/>
+      <c r="P3" s="13">
+        <v>48.0</v>
+      </c>
       <c r="Q3" s="13"/>
       <c r="R3" s="13"/>
       <c r="S3" s="13"/>
@@ -955,7 +964,9 @@
       <c r="O4" s="22">
         <v>0.5865</v>
       </c>
-      <c r="P4" s="22"/>
+      <c r="P4" s="22">
+        <v>0.5271</v>
+      </c>
       <c r="Q4" s="22"/>
       <c r="R4" s="22"/>
       <c r="S4" s="22"/>
@@ -1028,7 +1039,9 @@
       <c r="O5" s="13">
         <v>2.0</v>
       </c>
-      <c r="P5" s="13"/>
+      <c r="P5" s="13">
+        <v>2.0</v>
+      </c>
       <c r="Q5" s="13"/>
       <c r="R5" s="13"/>
       <c r="S5" s="13"/>
@@ -1101,7 +1114,9 @@
       <c r="O6" s="13">
         <v>10.0</v>
       </c>
-      <c r="P6" s="26"/>
+      <c r="P6" s="13">
+        <v>10.0</v>
+      </c>
       <c r="Q6" s="26"/>
       <c r="R6" s="26"/>
       <c r="S6" s="26"/>
@@ -1174,7 +1189,9 @@
       <c r="O7" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="P7" s="26"/>
+      <c r="P7" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="Q7" s="26"/>
       <c r="R7" s="26"/>
       <c r="S7" s="26"/>
@@ -1247,7 +1264,9 @@
       <c r="O8" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="P8" s="26"/>
+      <c r="P8" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="Q8" s="26"/>
       <c r="R8" s="26"/>
       <c r="S8" s="26"/>
@@ -1320,7 +1339,9 @@
       <c r="O9" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="P9" s="26"/>
+      <c r="P9" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="Q9" s="26"/>
       <c r="R9" s="26"/>
       <c r="S9" s="26"/>
@@ -1393,7 +1414,9 @@
       <c r="O10" s="31">
         <v>0.28</v>
       </c>
-      <c r="P10" s="13"/>
+      <c r="P10" s="31">
+        <v>0.28</v>
+      </c>
       <c r="Q10" s="13"/>
       <c r="R10" s="13"/>
       <c r="S10" s="13"/>
@@ -1466,7 +1489,9 @@
       <c r="O11" s="13">
         <v>36.0</v>
       </c>
-      <c r="P11" s="13"/>
+      <c r="P11" s="13">
+        <v>36.0</v>
+      </c>
       <c r="Q11" s="13"/>
       <c r="R11" s="13"/>
       <c r="S11" s="13"/>
@@ -1539,7 +1564,9 @@
       <c r="O12" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="P12" s="13"/>
+      <c r="P12" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="Q12" s="13"/>
       <c r="R12" s="13"/>
       <c r="S12" s="13"/>
@@ -1606,13 +1633,15 @@
       <c r="M13" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="N13" s="13" t="s">
+      <c r="N13" s="33" t="s">
         <v>31</v>
       </c>
-      <c r="O13" s="13" t="s">
+      <c r="O13" s="33" t="s">
         <v>32</v>
       </c>
-      <c r="P13" s="13"/>
+      <c r="P13" s="33" t="s">
+        <v>33</v>
+      </c>
       <c r="Q13" s="13"/>
       <c r="R13" s="13"/>
       <c r="S13" s="13"/>
@@ -1644,7 +1673,7 @@
     <row r="14">
       <c r="A14" s="14"/>
       <c r="B14" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C14" s="9">
         <v>0.0</v>
@@ -1685,7 +1714,9 @@
       <c r="O14" s="12">
         <v>0.0</v>
       </c>
-      <c r="P14" s="26"/>
+      <c r="P14" s="12">
+        <v>0.0</v>
+      </c>
       <c r="Q14" s="26"/>
       <c r="R14" s="26"/>
       <c r="S14" s="26"/>
@@ -1716,10 +1747,10 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>13</v>
@@ -1760,7 +1791,9 @@
       <c r="O15" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="P15" s="13"/>
+      <c r="P15" s="12">
+        <v>2.0</v>
+      </c>
       <c r="Q15" s="13"/>
       <c r="R15" s="13"/>
       <c r="S15" s="13"/>
@@ -1792,7 +1825,7 @@
     <row r="16">
       <c r="A16" s="14"/>
       <c r="B16" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>13</v>
@@ -1833,7 +1866,9 @@
       <c r="O16" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="P16" s="13"/>
+      <c r="P16" s="12" t="s">
+        <v>13</v>
+      </c>
       <c r="Q16" s="13"/>
       <c r="R16" s="13"/>
       <c r="S16" s="13"/>
@@ -1864,51 +1899,53 @@
     </row>
     <row r="17">
       <c r="A17" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G17" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H17" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I17" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J17" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K17" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L17" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M17" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N17" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="O17" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
-      <c r="P17" s="13"/>
+      <c r="P17" s="39" t="s">
+        <v>40</v>
+      </c>
       <c r="Q17" s="13"/>
       <c r="R17" s="13"/>
       <c r="S17" s="13"/>
@@ -1940,48 +1977,50 @@
     <row r="18">
       <c r="A18" s="14"/>
       <c r="B18" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="9" t="s">
-        <v>39</v>
-      </c>
       <c r="D18" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G18" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H18" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I18" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J18" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K18" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L18" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M18" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N18" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="O18" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
-      <c r="P18" s="26"/>
+      <c r="P18" s="39" t="s">
+        <v>40</v>
+      </c>
       <c r="Q18" s="26"/>
       <c r="R18" s="26"/>
       <c r="S18" s="26"/>
@@ -2013,48 +2052,50 @@
     <row r="19">
       <c r="A19" s="14"/>
       <c r="B19" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G19" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H19" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I19" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J19" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K19" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L19" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M19" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N19" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="O19" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
-      <c r="P19" s="26"/>
+      <c r="P19" s="39" t="s">
+        <v>40</v>
+      </c>
       <c r="Q19" s="26"/>
       <c r="R19" s="26"/>
       <c r="S19" s="26"/>
@@ -2086,48 +2127,50 @@
     <row r="20">
       <c r="A20" s="14"/>
       <c r="B20" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G20" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H20" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I20" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J20" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K20" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L20" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M20" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N20" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="O20" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
-      <c r="P20" s="26"/>
+      <c r="P20" s="39" t="s">
+        <v>40</v>
+      </c>
       <c r="Q20" s="26"/>
       <c r="R20" s="26"/>
       <c r="S20" s="26"/>
@@ -2158,51 +2201,53 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G21" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="H21" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I21" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J21" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="K21" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L21" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="M21" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="N21" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="O21" s="39" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
-      <c r="P21" s="13"/>
+      <c r="P21" s="39" t="s">
+        <v>40</v>
+      </c>
       <c r="Q21" s="13"/>
       <c r="R21" s="13"/>
       <c r="S21" s="13"/>
@@ -2234,7 +2279,7 @@
     <row r="22">
       <c r="A22" s="14"/>
       <c r="B22" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C22" s="9"/>
       <c r="D22" s="10"/>
@@ -2249,7 +2294,7 @@
       <c r="M22" s="12"/>
       <c r="N22" s="12"/>
       <c r="O22" s="12"/>
-      <c r="P22" s="26"/>
+      <c r="P22" s="12"/>
       <c r="Q22" s="26"/>
       <c r="R22" s="26"/>
       <c r="S22" s="26"/>
@@ -2281,7 +2326,7 @@
     <row r="23">
       <c r="A23" s="14"/>
       <c r="B23" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C23" s="9"/>
       <c r="D23" s="10"/>
@@ -2328,7 +2373,7 @@
     <row r="24">
       <c r="A24" s="14"/>
       <c r="B24" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C24" s="9"/>
       <c r="D24" s="10"/>
@@ -2343,7 +2388,7 @@
       <c r="M24" s="13"/>
       <c r="N24" s="13"/>
       <c r="O24" s="13"/>
-      <c r="P24" s="26"/>
+      <c r="P24" s="13"/>
       <c r="Q24" s="26"/>
       <c r="R24" s="26"/>
       <c r="S24" s="26"/>
@@ -2374,10 +2419,10 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="10"/>
@@ -2392,7 +2437,7 @@
       <c r="M25" s="13"/>
       <c r="N25" s="13"/>
       <c r="O25" s="13"/>
-      <c r="P25" s="26"/>
+      <c r="P25" s="13"/>
       <c r="Q25" s="26"/>
       <c r="R25" s="26"/>
       <c r="S25" s="26"/>
@@ -2424,7 +2469,7 @@
     <row r="26">
       <c r="A26" s="14"/>
       <c r="B26" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C26" s="9"/>
       <c r="D26" s="10"/>
@@ -2439,7 +2484,7 @@
       <c r="M26" s="13"/>
       <c r="N26" s="13"/>
       <c r="O26" s="13"/>
-      <c r="P26" s="26"/>
+      <c r="P26" s="13"/>
       <c r="Q26" s="26"/>
       <c r="R26" s="26"/>
       <c r="S26" s="26"/>
@@ -2471,7 +2516,7 @@
     <row r="27">
       <c r="A27" s="14"/>
       <c r="B27" s="8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C27" s="9"/>
       <c r="D27" s="10"/>
@@ -2486,7 +2531,7 @@
       <c r="M27" s="13"/>
       <c r="N27" s="13"/>
       <c r="O27" s="13"/>
-      <c r="P27" s="26"/>
+      <c r="P27" s="13"/>
       <c r="Q27" s="26"/>
       <c r="R27" s="26"/>
       <c r="S27" s="26"/>
@@ -2518,7 +2563,7 @@
     <row r="28">
       <c r="A28" s="45"/>
       <c r="B28" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C28" s="9"/>
       <c r="D28" s="10"/>
@@ -2533,7 +2578,7 @@
       <c r="M28" s="13"/>
       <c r="N28" s="13"/>
       <c r="O28" s="13"/>
-      <c r="P28" s="26"/>
+      <c r="P28" s="13"/>
       <c r="Q28" s="26"/>
       <c r="R28" s="26"/>
       <c r="S28" s="26"/>

</xml_diff>

<commit_message>
chore: sync latest live master data and metrics
</commit_message>
<xml_diff>
--- a/public/master/KPI _ Automation COE (2).xlsx
+++ b/public/master/KPI _ Automation COE (2).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="54">
   <si>
     <t>Category</t>
   </si>
@@ -113,6 +113,9 @@
   </si>
   <si>
     <t>492 (279, 213)</t>
+  </si>
+  <si>
+    <t>515 (299, 216)</t>
   </si>
   <si>
     <t>AI Search</t>
@@ -740,7 +743,9 @@
       <c r="P1" s="3">
         <v>46297.0</v>
       </c>
-      <c r="Q1" s="5"/>
+      <c r="Q1" s="3">
+        <v>46304.0</v>
+      </c>
       <c r="R1" s="5"/>
       <c r="S1" s="5"/>
       <c r="T1" s="5"/>
@@ -817,7 +822,9 @@
       <c r="P2" s="13">
         <v>292.0</v>
       </c>
-      <c r="Q2" s="13"/>
+      <c r="Q2" s="13">
+        <v>362.0</v>
+      </c>
       <c r="R2" s="13"/>
       <c r="S2" s="13"/>
       <c r="T2" s="13"/>
@@ -892,7 +899,9 @@
       <c r="P3" s="13">
         <v>48.0</v>
       </c>
-      <c r="Q3" s="13"/>
+      <c r="Q3" s="13">
+        <v>77.0</v>
+      </c>
       <c r="R3" s="13"/>
       <c r="S3" s="13"/>
       <c r="T3" s="13"/>
@@ -967,7 +976,9 @@
       <c r="P4" s="22">
         <v>0.5271</v>
       </c>
-      <c r="Q4" s="22"/>
+      <c r="Q4" s="22">
+        <v>0.5473</v>
+      </c>
       <c r="R4" s="22"/>
       <c r="S4" s="22"/>
       <c r="T4" s="22"/>
@@ -1042,7 +1053,9 @@
       <c r="P5" s="13">
         <v>2.0</v>
       </c>
-      <c r="Q5" s="13"/>
+      <c r="Q5" s="13">
+        <v>2.0</v>
+      </c>
       <c r="R5" s="13"/>
       <c r="S5" s="13"/>
       <c r="T5" s="13"/>
@@ -1117,7 +1130,9 @@
       <c r="P6" s="13">
         <v>10.0</v>
       </c>
-      <c r="Q6" s="26"/>
+      <c r="Q6" s="13">
+        <v>10.0</v>
+      </c>
       <c r="R6" s="26"/>
       <c r="S6" s="26"/>
       <c r="T6" s="26"/>
@@ -1192,7 +1207,9 @@
       <c r="P7" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="Q7" s="26"/>
+      <c r="Q7" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="R7" s="26"/>
       <c r="S7" s="26"/>
       <c r="T7" s="26"/>
@@ -1267,7 +1284,9 @@
       <c r="P8" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="Q8" s="26"/>
+      <c r="Q8" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="R8" s="26"/>
       <c r="S8" s="26"/>
       <c r="T8" s="26"/>
@@ -1342,7 +1361,9 @@
       <c r="P9" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="Q9" s="26"/>
+      <c r="Q9" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="R9" s="26"/>
       <c r="S9" s="26"/>
       <c r="T9" s="26"/>
@@ -1417,7 +1438,9 @@
       <c r="P10" s="31">
         <v>0.28</v>
       </c>
-      <c r="Q10" s="13"/>
+      <c r="Q10" s="31">
+        <v>0.28</v>
+      </c>
       <c r="R10" s="13"/>
       <c r="S10" s="13"/>
       <c r="T10" s="13"/>
@@ -1492,7 +1515,9 @@
       <c r="P11" s="13">
         <v>36.0</v>
       </c>
-      <c r="Q11" s="13"/>
+      <c r="Q11" s="13">
+        <v>36.0</v>
+      </c>
       <c r="R11" s="13"/>
       <c r="S11" s="13"/>
       <c r="T11" s="13"/>
@@ -1567,7 +1592,9 @@
       <c r="P12" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="Q12" s="13"/>
+      <c r="Q12" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="R12" s="13"/>
       <c r="S12" s="13"/>
       <c r="T12" s="13"/>
@@ -1642,7 +1669,9 @@
       <c r="P13" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="Q13" s="13"/>
+      <c r="Q13" s="33" t="s">
+        <v>34</v>
+      </c>
       <c r="R13" s="13"/>
       <c r="S13" s="13"/>
       <c r="T13" s="13"/>
@@ -1673,7 +1702,7 @@
     <row r="14">
       <c r="A14" s="14"/>
       <c r="B14" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C14" s="9">
         <v>0.0</v>
@@ -1717,7 +1746,9 @@
       <c r="P14" s="12">
         <v>0.0</v>
       </c>
-      <c r="Q14" s="26"/>
+      <c r="Q14" s="12">
+        <v>0.0</v>
+      </c>
       <c r="R14" s="26"/>
       <c r="S14" s="26"/>
       <c r="T14" s="26"/>
@@ -1747,10 +1778,10 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>13</v>
@@ -1794,7 +1825,9 @@
       <c r="P15" s="12">
         <v>2.0</v>
       </c>
-      <c r="Q15" s="13"/>
+      <c r="Q15" s="12">
+        <v>3.0</v>
+      </c>
       <c r="R15" s="13"/>
       <c r="S15" s="13"/>
       <c r="T15" s="26"/>
@@ -1825,7 +1858,7 @@
     <row r="16">
       <c r="A16" s="14"/>
       <c r="B16" s="8" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>13</v>
@@ -1869,7 +1902,9 @@
       <c r="P16" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="Q16" s="13"/>
+      <c r="Q16" s="12" t="s">
+        <v>13</v>
+      </c>
       <c r="R16" s="13"/>
       <c r="S16" s="13"/>
       <c r="T16" s="26"/>
@@ -1899,54 +1934,56 @@
     </row>
     <row r="17">
       <c r="A17" s="7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G17" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H17" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I17" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J17" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K17" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L17" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M17" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N17" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="O17" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P17" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
-      <c r="Q17" s="13"/>
+      <c r="Q17" s="39" t="s">
+        <v>41</v>
+      </c>
       <c r="R17" s="13"/>
       <c r="S17" s="13"/>
       <c r="T17" s="13"/>
@@ -1977,51 +2014,53 @@
     <row r="18">
       <c r="A18" s="14"/>
       <c r="B18" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C18" s="9" t="s">
-        <v>40</v>
-      </c>
       <c r="D18" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G18" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H18" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I18" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J18" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K18" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L18" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M18" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N18" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="O18" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P18" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
-      <c r="Q18" s="26"/>
+      <c r="Q18" s="39" t="s">
+        <v>41</v>
+      </c>
       <c r="R18" s="26"/>
       <c r="S18" s="26"/>
       <c r="T18" s="26"/>
@@ -2052,51 +2091,53 @@
     <row r="19">
       <c r="A19" s="14"/>
       <c r="B19" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G19" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H19" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I19" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J19" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K19" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L19" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M19" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N19" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="O19" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P19" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
-      <c r="Q19" s="26"/>
+      <c r="Q19" s="39" t="s">
+        <v>41</v>
+      </c>
       <c r="R19" s="26"/>
       <c r="S19" s="26"/>
       <c r="T19" s="26"/>
@@ -2127,51 +2168,53 @@
     <row r="20">
       <c r="A20" s="14"/>
       <c r="B20" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G20" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H20" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I20" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J20" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K20" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L20" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M20" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N20" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="O20" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P20" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
-      <c r="Q20" s="26"/>
+      <c r="Q20" s="39" t="s">
+        <v>41</v>
+      </c>
       <c r="R20" s="26"/>
       <c r="S20" s="26"/>
       <c r="T20" s="26"/>
@@ -2201,54 +2244,56 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G21" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H21" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I21" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J21" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K21" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L21" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="M21" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="N21" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="O21" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="P21" s="39" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
-      <c r="Q21" s="13"/>
+      <c r="Q21" s="39" t="s">
+        <v>41</v>
+      </c>
       <c r="R21" s="13"/>
       <c r="S21" s="13"/>
       <c r="T21" s="13"/>
@@ -2279,7 +2324,7 @@
     <row r="22">
       <c r="A22" s="14"/>
       <c r="B22" s="8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C22" s="9"/>
       <c r="D22" s="10"/>
@@ -2295,7 +2340,7 @@
       <c r="N22" s="12"/>
       <c r="O22" s="12"/>
       <c r="P22" s="12"/>
-      <c r="Q22" s="26"/>
+      <c r="Q22" s="12"/>
       <c r="R22" s="26"/>
       <c r="S22" s="26"/>
       <c r="T22" s="26"/>
@@ -2326,7 +2371,7 @@
     <row r="23">
       <c r="A23" s="14"/>
       <c r="B23" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C23" s="9"/>
       <c r="D23" s="10"/>
@@ -2373,7 +2418,7 @@
     <row r="24">
       <c r="A24" s="14"/>
       <c r="B24" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C24" s="9"/>
       <c r="D24" s="10"/>
@@ -2389,7 +2434,7 @@
       <c r="N24" s="13"/>
       <c r="O24" s="13"/>
       <c r="P24" s="13"/>
-      <c r="Q24" s="26"/>
+      <c r="Q24" s="13"/>
       <c r="R24" s="26"/>
       <c r="S24" s="26"/>
       <c r="T24" s="26"/>
@@ -2419,10 +2464,10 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="10"/>
@@ -2438,7 +2483,7 @@
       <c r="N25" s="13"/>
       <c r="O25" s="13"/>
       <c r="P25" s="13"/>
-      <c r="Q25" s="26"/>
+      <c r="Q25" s="13"/>
       <c r="R25" s="26"/>
       <c r="S25" s="26"/>
       <c r="T25" s="26"/>
@@ -2469,7 +2514,7 @@
     <row r="26">
       <c r="A26" s="14"/>
       <c r="B26" s="8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C26" s="9"/>
       <c r="D26" s="10"/>
@@ -2485,7 +2530,7 @@
       <c r="N26" s="13"/>
       <c r="O26" s="13"/>
       <c r="P26" s="13"/>
-      <c r="Q26" s="26"/>
+      <c r="Q26" s="13"/>
       <c r="R26" s="26"/>
       <c r="S26" s="26"/>
       <c r="T26" s="26"/>
@@ -2516,7 +2561,7 @@
     <row r="27">
       <c r="A27" s="14"/>
       <c r="B27" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C27" s="9"/>
       <c r="D27" s="10"/>
@@ -2532,7 +2577,7 @@
       <c r="N27" s="13"/>
       <c r="O27" s="13"/>
       <c r="P27" s="13"/>
-      <c r="Q27" s="26"/>
+      <c r="Q27" s="13"/>
       <c r="R27" s="26"/>
       <c r="S27" s="26"/>
       <c r="T27" s="26"/>
@@ -2563,7 +2608,7 @@
     <row r="28">
       <c r="A28" s="45"/>
       <c r="B28" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C28" s="9"/>
       <c r="D28" s="10"/>
@@ -2579,7 +2624,7 @@
       <c r="N28" s="13"/>
       <c r="O28" s="13"/>
       <c r="P28" s="13"/>
-      <c r="Q28" s="26"/>
+      <c r="Q28" s="13"/>
       <c r="R28" s="26"/>
       <c r="S28" s="26"/>
       <c r="T28" s="26"/>

</xml_diff>

<commit_message>
fix: resolve Google Sheet sync button to dynamically extract 17 weeks up to 23-Oct with proxy fallback
</commit_message>
<xml_diff>
--- a/public/master/KPI _ Automation COE (2).xlsx
+++ b/public/master/KPI _ Automation COE (2).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="56">
   <si>
     <t>Category</t>
   </si>
@@ -119,6 +119,9 @@
   </si>
   <si>
     <t>556 (337, 219)</t>
+  </si>
+  <si>
+    <t>584 (342, 242)</t>
   </si>
   <si>
     <t>AI Search</t>
@@ -755,7 +758,9 @@
       <c r="R1" s="3">
         <v>46311.0</v>
       </c>
-      <c r="S1" s="5"/>
+      <c r="S1" s="3">
+        <v>46318.0</v>
+      </c>
       <c r="T1" s="5"/>
       <c r="U1" s="5"/>
       <c r="V1" s="5"/>
@@ -836,7 +841,9 @@
       <c r="R2" s="13">
         <v>277.0</v>
       </c>
-      <c r="S2" s="13"/>
+      <c r="S2" s="13">
+        <v>225.0</v>
+      </c>
       <c r="T2" s="13"/>
       <c r="U2" s="13"/>
       <c r="V2" s="13"/>
@@ -915,7 +922,9 @@
       <c r="R3" s="13">
         <v>51.0</v>
       </c>
-      <c r="S3" s="13"/>
+      <c r="S3" s="13">
+        <v>60.0</v>
+      </c>
       <c r="T3" s="13"/>
       <c r="U3" s="13"/>
       <c r="V3" s="13"/>
@@ -994,7 +1003,9 @@
       <c r="R4" s="22">
         <v>0.4867</v>
       </c>
-      <c r="S4" s="22"/>
+      <c r="S4" s="22">
+        <v>0.5238</v>
+      </c>
       <c r="T4" s="22"/>
       <c r="U4" s="22"/>
       <c r="V4" s="22"/>
@@ -1073,7 +1084,9 @@
       <c r="R5" s="13">
         <v>2.0</v>
       </c>
-      <c r="S5" s="13"/>
+      <c r="S5" s="13">
+        <v>2.0</v>
+      </c>
       <c r="T5" s="13"/>
       <c r="U5" s="13"/>
       <c r="V5" s="13"/>
@@ -1152,7 +1165,9 @@
       <c r="R6" s="13">
         <v>10.0</v>
       </c>
-      <c r="S6" s="26"/>
+      <c r="S6" s="13">
+        <v>10.0</v>
+      </c>
       <c r="T6" s="26"/>
       <c r="U6" s="26"/>
       <c r="V6" s="26"/>
@@ -1231,7 +1246,9 @@
       <c r="R7" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="S7" s="26"/>
+      <c r="S7" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="T7" s="26"/>
       <c r="U7" s="26"/>
       <c r="V7" s="26"/>
@@ -1310,7 +1327,9 @@
       <c r="R8" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="S8" s="26"/>
+      <c r="S8" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="T8" s="26"/>
       <c r="U8" s="26"/>
       <c r="V8" s="26"/>
@@ -1389,7 +1408,9 @@
       <c r="R9" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="S9" s="26"/>
+      <c r="S9" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="T9" s="26"/>
       <c r="U9" s="26"/>
       <c r="V9" s="26"/>
@@ -1468,7 +1489,9 @@
       <c r="R10" s="31">
         <v>0.28</v>
       </c>
-      <c r="S10" s="13"/>
+      <c r="S10" s="31">
+        <v>0.28</v>
+      </c>
       <c r="T10" s="13"/>
       <c r="U10" s="13"/>
       <c r="V10" s="13"/>
@@ -1547,7 +1570,9 @@
       <c r="R11" s="13">
         <v>36.0</v>
       </c>
-      <c r="S11" s="13"/>
+      <c r="S11" s="13">
+        <v>36.0</v>
+      </c>
       <c r="T11" s="13"/>
       <c r="U11" s="13"/>
       <c r="V11" s="13"/>
@@ -1626,7 +1651,9 @@
       <c r="R12" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="S12" s="13"/>
+      <c r="S12" s="13" t="s">
+        <v>13</v>
+      </c>
       <c r="T12" s="13"/>
       <c r="U12" s="13"/>
       <c r="V12" s="13"/>
@@ -1705,7 +1732,9 @@
       <c r="R13" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="S13" s="13"/>
+      <c r="S13" s="33" t="s">
+        <v>36</v>
+      </c>
       <c r="T13" s="13"/>
       <c r="U13" s="13"/>
       <c r="V13" s="13"/>
@@ -1734,7 +1763,7 @@
     <row r="14">
       <c r="A14" s="14"/>
       <c r="B14" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C14" s="9">
         <v>0.0</v>
@@ -1784,7 +1813,9 @@
       <c r="R14" s="12">
         <v>0.0</v>
       </c>
-      <c r="S14" s="26"/>
+      <c r="S14" s="12">
+        <v>0.0</v>
+      </c>
       <c r="T14" s="26"/>
       <c r="U14" s="26"/>
       <c r="V14" s="26"/>
@@ -1812,10 +1843,10 @@
     </row>
     <row r="15">
       <c r="A15" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C15" s="9" t="s">
         <v>13</v>
@@ -1865,7 +1896,9 @@
       <c r="R15" s="12">
         <v>1.0</v>
       </c>
-      <c r="S15" s="13"/>
+      <c r="S15" s="12">
+        <v>2.0</v>
+      </c>
       <c r="T15" s="26"/>
       <c r="U15" s="26"/>
       <c r="V15" s="26"/>
@@ -1894,7 +1927,7 @@
     <row r="16">
       <c r="A16" s="14"/>
       <c r="B16" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C16" s="9" t="s">
         <v>13</v>
@@ -1944,7 +1977,9 @@
       <c r="R16" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="S16" s="13"/>
+      <c r="S16" s="12" t="s">
+        <v>13</v>
+      </c>
       <c r="T16" s="26"/>
       <c r="U16" s="26"/>
       <c r="V16" s="26"/>
@@ -1972,60 +2007,62 @@
     </row>
     <row r="17">
       <c r="A17" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G17" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H17" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I17" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J17" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K17" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L17" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M17" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N17" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="O17" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P17" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q17" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="R17" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
-      <c r="S17" s="13"/>
+      <c r="S17" s="39" t="s">
+        <v>43</v>
+      </c>
       <c r="T17" s="13"/>
       <c r="U17" s="13"/>
       <c r="V17" s="13"/>
@@ -2054,57 +2091,59 @@
     <row r="18">
       <c r="A18" s="14"/>
       <c r="B18" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="9" t="s">
-        <v>42</v>
-      </c>
       <c r="D18" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G18" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H18" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I18" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J18" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K18" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L18" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M18" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N18" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="O18" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P18" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q18" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="R18" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
-      <c r="S18" s="26"/>
+      <c r="S18" s="39" t="s">
+        <v>43</v>
+      </c>
       <c r="T18" s="26"/>
       <c r="U18" s="26"/>
       <c r="V18" s="41"/>
@@ -2133,57 +2172,59 @@
     <row r="19">
       <c r="A19" s="14"/>
       <c r="B19" s="8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G19" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H19" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I19" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J19" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K19" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L19" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M19" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N19" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="O19" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P19" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q19" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="R19" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
-      <c r="S19" s="26"/>
+      <c r="S19" s="39" t="s">
+        <v>43</v>
+      </c>
       <c r="T19" s="26"/>
       <c r="U19" s="26"/>
       <c r="V19" s="40"/>
@@ -2212,57 +2253,59 @@
     <row r="20">
       <c r="A20" s="14"/>
       <c r="B20" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G20" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H20" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I20" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J20" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K20" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L20" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M20" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N20" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="O20" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P20" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q20" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="R20" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
-      <c r="S20" s="26"/>
+      <c r="S20" s="39" t="s">
+        <v>43</v>
+      </c>
       <c r="T20" s="26"/>
       <c r="U20" s="26"/>
       <c r="V20" s="40"/>
@@ -2290,52 +2333,52 @@
     </row>
     <row r="21">
       <c r="A21" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G21" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H21" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I21" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J21" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K21" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L21" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M21" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="N21" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="O21" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="P21" s="39" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="Q21" s="44">
         <v>1.0</v>
@@ -2343,7 +2386,9 @@
       <c r="R21" s="44">
         <v>2.0</v>
       </c>
-      <c r="S21" s="13"/>
+      <c r="S21" s="44">
+        <v>2.0</v>
+      </c>
       <c r="T21" s="13"/>
       <c r="U21" s="13"/>
       <c r="V21" s="13"/>
@@ -2372,7 +2417,7 @@
     <row r="22">
       <c r="A22" s="14"/>
       <c r="B22" s="8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C22" s="9"/>
       <c r="D22" s="10"/>
@@ -2390,7 +2435,7 @@
       <c r="P22" s="12"/>
       <c r="Q22" s="12"/>
       <c r="R22" s="12"/>
-      <c r="S22" s="26"/>
+      <c r="S22" s="12"/>
       <c r="T22" s="26"/>
       <c r="U22" s="26"/>
       <c r="V22" s="26"/>
@@ -2419,7 +2464,7 @@
     <row r="23">
       <c r="A23" s="14"/>
       <c r="B23" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C23" s="9"/>
       <c r="D23" s="10"/>
@@ -2466,7 +2511,7 @@
     <row r="24">
       <c r="A24" s="14"/>
       <c r="B24" s="8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C24" s="9"/>
       <c r="D24" s="10"/>
@@ -2484,7 +2529,7 @@
       <c r="P24" s="13"/>
       <c r="Q24" s="13"/>
       <c r="R24" s="13"/>
-      <c r="S24" s="26"/>
+      <c r="S24" s="13"/>
       <c r="T24" s="26"/>
       <c r="U24" s="26"/>
       <c r="V24" s="26"/>
@@ -2512,10 +2557,10 @@
     </row>
     <row r="25">
       <c r="A25" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="10"/>
@@ -2533,7 +2578,7 @@
       <c r="P25" s="13"/>
       <c r="Q25" s="13"/>
       <c r="R25" s="13"/>
-      <c r="S25" s="26"/>
+      <c r="S25" s="13"/>
       <c r="T25" s="26"/>
       <c r="U25" s="26"/>
       <c r="V25" s="26"/>
@@ -2562,7 +2607,7 @@
     <row r="26">
       <c r="A26" s="14"/>
       <c r="B26" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C26" s="9"/>
       <c r="D26" s="10"/>
@@ -2580,7 +2625,7 @@
       <c r="P26" s="13"/>
       <c r="Q26" s="13"/>
       <c r="R26" s="13"/>
-      <c r="S26" s="26"/>
+      <c r="S26" s="13"/>
       <c r="T26" s="26"/>
       <c r="U26" s="26"/>
       <c r="V26" s="26"/>
@@ -2609,7 +2654,7 @@
     <row r="27">
       <c r="A27" s="14"/>
       <c r="B27" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C27" s="9"/>
       <c r="D27" s="10"/>
@@ -2627,7 +2672,7 @@
       <c r="P27" s="13"/>
       <c r="Q27" s="13"/>
       <c r="R27" s="13"/>
-      <c r="S27" s="26"/>
+      <c r="S27" s="13"/>
       <c r="T27" s="26"/>
       <c r="U27" s="26"/>
       <c r="V27" s="26"/>
@@ -2656,7 +2701,7 @@
     <row r="28">
       <c r="A28" s="46"/>
       <c r="B28" s="8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C28" s="9"/>
       <c r="D28" s="10"/>
@@ -2674,7 +2719,7 @@
       <c r="P28" s="13"/>
       <c r="Q28" s="13"/>
       <c r="R28" s="13"/>
-      <c r="S28" s="26"/>
+      <c r="S28" s="13"/>
       <c r="T28" s="26"/>
       <c r="U28" s="26"/>
       <c r="V28" s="26"/>

</xml_diff>